<commit_message>
Auto update Pengadaan 2026-10-28 10:10:46
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-28).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-28).xlsx
@@ -924,13 +924,13 @@
         <v>122</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>756952316</v>
+        <v>756952315</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F15" s="10" t="n">
-        <v>63250745</v>
+        <v>63250744</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>2</v>
@@ -1004,35 +1004,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1154,35 +1146,27 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E20" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G20" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>1193100910</v>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
@@ -1308,13 +1292,13 @@
         <v>93</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1145584728</v>
+        <v>1148350728</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>55769294</v>
+        <v>58535294</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>6</v>
@@ -1339,22 +1323,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>414639535</v>
+        <v>403884747</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>84907554</v>
+        <v>74152766</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>78869208</v>
+        <v>128214258</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>62</v>
@@ -1373,22 +1357,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>896770286</v>
+        <v>895266732</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>137583844</v>
+        <v>136080290</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>116218702</v>
+        <v>1573507514</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>106</v>
@@ -1407,22 +1391,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>497942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>338050900</v>
+        <v>3037348900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1478,13 +1462,13 @@
         <v>100</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>901471767</v>
+        <v>891844767</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>5</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>77396400</v>
+        <v>67769400</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>5</v>
@@ -1509,16 +1493,16 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>2559551299</v>
+        <v>2550047146</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>58</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>1228508400</v>
+        <v>1219004247</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>58</v>
@@ -1527,7 +1511,7 @@
         <v>1207378630.6</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>1331042899</v>
@@ -1543,22 +1527,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>94495292</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>90557607</v>
+        <v>240557607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>42</v>
@@ -1580,13 +1564,13 @@
         <v>52</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>283301771</v>
+        <v>283157746</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>16</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>70581100</v>
+        <v>70437075</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>16</v>
@@ -1614,13 +1598,13 @@
         <v>113</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>767894130</v>
+        <v>764274671</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>12</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>169142604</v>
+        <v>165523145</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>12</v>
@@ -1648,13 +1632,13 @@
         <v>44</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>366634933</v>
+        <v>278301799</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>4</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>98994684</v>
+        <v>10661550</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>4</v>
@@ -1716,13 +1700,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>463972148</v>
+        <v>463836830</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>93366423</v>
+        <v>93231105</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1750,13 +1734,13 @@
         <v>73</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>763988281</v>
+        <v>763363033</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>13</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>334343818</v>
+        <v>333718570</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>13</v>
@@ -1781,28 +1765,28 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>1098424791</v>
+        <v>954862891</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>365576502</v>
+        <v>271204602</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>355577400</v>
+        <v>1186117670</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>732848289</v>
+        <v>683658289</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -1818,13 +1802,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>384332451</v>
+        <v>382731831</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>12</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>101993338</v>
+        <v>100392718</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>12</v>
@@ -1849,22 +1833,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>1262512215</v>
+        <v>1236982215</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>396795289</v>
+        <v>371265289</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>392670830</v>
+        <v>432747380</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>82</v>
@@ -1886,13 +1870,13 @@
         <v>83</v>
       </c>
       <c r="D40" s="9" t="n">
-        <v>956575994</v>
+        <v>953657184</v>
       </c>
       <c r="E40" s="7" t="n">
         <v>60</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>783150756</v>
+        <v>780231946</v>
       </c>
       <c r="G40" s="7" t="n">
         <v>60</v>
@@ -1988,13 +1972,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>708077545</v>
+        <v>727698127</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2019,22 +2003,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>340998868</v>
+        <v>270482868</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>151137140</v>
+        <v>80621140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>72726534</v>
+        <v>83626512</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>18</v>
@@ -2103,22 +2087,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1095276809</v>
+        <v>1143929219</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>124972901</v>
+        <v>173625311</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>121983128</v>
+        <v>318350703</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>160</v>
@@ -2224,13 +2208,13 @@
         <v>98</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>582264876</v>
+        <v>580339876</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>37</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>288710598</v>
+        <v>286785598</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>37</v>
@@ -2323,22 +2307,22 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F52" s="9" t="n">
         <v>24520790</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>22939000</v>
+        <v>88340200</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>10</v>
@@ -3108,13 +3092,13 @@
         <v>41</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>330321582</v>
+        <v>323431257</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>35716900</v>
+        <v>28826575</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3139,22 +3123,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>158730000</v>
+        <v>2359971000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3260,7 +3244,7 @@
         <v>112</v>
       </c>
       <c r="D75" s="10" t="n">
-        <v>1430349546</v>
+        <v>1395949546</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3278,7 +3262,7 @@
         <v>94</v>
       </c>
       <c r="J75" s="10" t="n">
-        <v>1010475360</v>
+        <v>976075360</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3294,13 +3278,13 @@
         <v>145</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1495157470</v>
+        <v>1487523470</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>24</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>207985114</v>
+        <v>200351114</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>24</v>
@@ -3323,28 +3307,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3960</v>
+        <v>4012</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>34325700842</v>
+        <v>33977516499</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>593</v>
+        <v>643</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>8030739773</v>
+        <v>7766145430</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>593</v>
+        <v>643</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>7470998070.6</v>
+        <v>18161057415.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3367</v>
+        <v>3369</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>26294961069</v>
+        <v>26211371069</v>
       </c>
     </row>
   </sheetData>
@@ -3765,13 +3749,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>428765330</v>
+        <v>413165330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4197,45 +4181,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4267,29 +4235,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>111200910</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>111200910</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -4512,34 +4496,50 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>323734637</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>54773006</v>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="K24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" s="9" t="n">
-        <v>49345050</v>
+        <v>268961631</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M24" s="7" t="n">
         <v>3</v>
@@ -4558,34 +4558,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>1836525942</v>
+        <v>1613577499</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>1225542538</v>
+        <v>1002594095</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>896262562</v>
+        <v>766571463</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>896262562</v>
+        <v>766571463</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>334523972</v>
+        <v>204832873</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>8</v>
@@ -4804,28 +4804,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>538286000</v>
+        <v>388286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
@@ -4857,13 +4857,13 @@
         <v>7</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>477133090</v>
+        <v>490395090</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>66310000</v>
+        <v>79572000</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
@@ -5053,13 +5053,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>1668288113</v>
+        <v>1667542131</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>886469138</v>
+        <v>885723156</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5103,13 +5103,13 @@
         <v>38</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>4988812982</v>
+        <v>4988396732</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>36</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>4775708657</v>
+        <v>4775292407</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>36</v>
@@ -5150,40 +5150,40 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>3302665552</v>
+        <v>2671677052</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>1932930451</v>
+        <v>1487941951</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1837755163</v>
+        <v>1444011523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1581713573</v>
+        <v>1234505573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L37" s="10" t="n">
-        <v>713727983</v>
+        <v>366519983</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N37" s="10" t="n">
-        <v>1369735101</v>
+        <v>1183735101</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -5258,28 +5258,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>4655680948</v>
+        <v>4402582653</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>3041384586</v>
+        <v>2788286291</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2978771243</v>
+        <v>2753724693</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2804094693</v>
+        <v>2619124693</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>1</v>
@@ -5524,28 +5524,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>547117650</v>
+        <v>475135300</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K44" s="7" t="n">
         <v>2</v>
@@ -5640,28 +5640,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>932380105</v>
+        <v>716222170</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>471330601</v>
+        <v>255172666</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>448555830</v>
+        <v>252188255</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>309615830</v>
+        <v>113248255</v>
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
@@ -5996,34 +5996,38 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>559836352</v>
+        <v>319983894</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" s="9" t="n">
-        <v>301830114</v>
+        <v>61977656</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>68020787</v>
+        <v>2619587</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="K52" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="L52" s="9" t="n">
-        <v>65401200</v>
+        <v>2619587</v>
+      </c>
+      <c r="K52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M52" s="7" t="n">
         <v>3</v>
@@ -7165,13 +7169,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>423288615</v>
+        <v>392285593</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7432,28 +7436,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>3401653729</v>
+        <v>3551653729</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>564698247</v>
+        <v>714698247</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -7480,40 +7484,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>902</v>
+        <v>884</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>106666876710</v>
+        <v>105029650969</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>531</v>
+        <v>514</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>66581432351</v>
+        <v>65130206610</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>531</v>
+        <v>514</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64850492057.41</v>
+        <v>63867374555.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>390</v>
+        <v>375</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>49376647618.03</v>
+        <v>48480142306.03</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>1985506795</v>
+        <v>1393861446</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>40085444359</v>
+        <v>39899444359</v>
       </c>
     </row>
   </sheetData>
@@ -8323,28 +8327,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>26641091741</v>
+        <v>24844591741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>26641091741</v>
+        <v>24844591741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8430,29 +8434,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8484,29 +8504,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>1081900000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>1081900000</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -8542,13 +8578,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8596,7 +8632,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
@@ -8642,7 +8678,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8775,40 +8811,40 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>49096492181</v>
+        <v>6460249182</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>47632716881</v>
+        <v>4916473882</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2829407037</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2829407037</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>2945468782</v>
+        <v>1712457037</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N25" s="10" t="n">
-        <v>1463775300</v>
+        <v>1543775300</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -8995,10 +9031,10 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>13312906200</v>
+        <v>12978656340</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>23</v>
@@ -9029,10 +9065,10 @@
         </is>
       </c>
       <c r="M29" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N29" s="10" t="n">
-        <v>5252214356</v>
+        <v>4917964496</v>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -9408,13 +9444,13 @@
         <v>9</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>2208956507</v>
+        <v>2201730388</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>7</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>1763376386</v>
+        <v>1756150267</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>7</v>
@@ -9455,34 +9491,38 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>5765940896</v>
+        <v>4892340896</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>2946694000</v>
+        <v>2073094000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>2509890630</v>
+        <v>2073094000</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>2509890630</v>
-      </c>
-      <c r="K37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="10" t="n">
-        <v>436796630</v>
+        <v>2073094000</v>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9571,28 +9611,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>3813601480</v>
+        <v>3962367980</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>3013841480</v>
+        <v>3162607980</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>2</v>
@@ -9794,13 +9834,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11721,28 +11761,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>14398798637</v>
+        <v>7792798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>8054692000</v>
+        <v>1448692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -11933,28 +11973,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>7133067600</v>
+        <v>6783067600</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>3294207800</v>
+        <v>2944207800</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -11981,40 +12021,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>185102594591</v>
+        <v>131044499201</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>163</v>
+        <v>131</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>147660430043</v>
+        <v>93862084513</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>163</v>
+        <v>131</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71238198305.01001</v>
+        <v>64230554462.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>154</v>
+        <v>122</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>68978584305.01001</v>
+        <v>61970940462.01</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4633229261</v>
+        <v>2963420886</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>37442164548</v>
+        <v>37182414688</v>
       </c>
     </row>
   </sheetData>
@@ -13003,13 +13043,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13057,13 +13097,13 @@
         <v>1</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>5334500000</v>
+        <v>2646500000</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>5334500000</v>
+        <v>2646500000</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>1</v>
@@ -13458,28 +13498,40 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>5399320575</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>2700000000</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>2699298000</v>
-      </c>
-      <c r="I26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="9" t="n">
-        <v>2699298000</v>
+        <v>2699320575</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
@@ -16930,28 +16982,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>256072475553</v>
+        <v>250632775553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>149761870800</v>
+        <v>144322170800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>68536082008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>68536082008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>